<commit_message>
Update market making experiments: modify Excel file and remove temporary report document
</commit_message>
<xml_diff>
--- a/Excel/Market Making Experiments.xlsx
+++ b/Excel/Market Making Experiments.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zitangyu/Library/Mobile Documents/com~apple~CloudDocs/University/Extra/Research Projects/Quantitative Finance Projects/Market Making and Inventory Risk/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zitangyu/Library/Mobile Documents/com~apple~CloudDocs/University/Extra/Projects/Research Projects/Quantitative Finance Projects/Market Making and Inventory Risk/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62F641A-4B3B-C446-B721-3ADD48910928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFEE215-CB63-EA43-91F2-D845C4E0018C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10480" yWindow="600" windowWidth="30240" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -754,11 +754,11 @@
     <xf numFmtId="165" fontId="33" fillId="9" borderId="9" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="33" fillId="9" borderId="9" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="33" fillId="9" borderId="9" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="37" fillId="11" borderId="10" xfId="8"/>
-    <xf numFmtId="2" fontId="37" fillId="11" borderId="10" xfId="8" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="39" fillId="11" borderId="10" xfId="8" applyFont="1"/>
-    <xf numFmtId="166" fontId="38" fillId="11" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="38" fillId="11" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="10" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="37" fillId="11" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="39" fillId="11" borderId="10" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="38" fillId="11" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="38" fillId="11" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2622,21 +2622,21 @@
         <f>F2+Parameters!$B$3</f>
         <v>101</v>
       </c>
-      <c r="I2" s="2" t="str">
+      <c r="I2" s="2">
         <f t="shared" ref="I2:I21" ca="1" si="0">IF(P2&lt;&gt;"EXECUTED","",IF(B2="SELL",G2,H2))</f>
-        <v/>
+        <v>99</v>
       </c>
       <c r="J2" s="2">
         <f ca="1">IF(P2&lt;&gt;"EXECUTED",Parameters!$B$5,IF(B2="SELL",Parameters!$B$5-I2,Parameters!$B$5+I2))</f>
-        <v>0</v>
+        <v>-99</v>
       </c>
       <c r="K2" s="3">
         <f t="shared" ref="K2:K21" ca="1" si="1">IF(P2&lt;&gt;"EXECUTED",E2,IF(B2="SELL",E2+1,E2-1))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="2">
         <f t="shared" ref="L2:L21" ca="1" si="2">J2+K2*C2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" s="4">
         <f>MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C2-F2)))</f>
@@ -2648,7 +2648,7 @@
       <c r="O2" s="17"/>
       <c r="P2" s="45" t="str">
         <f ca="1">IF(R2&gt;Q2,"NO TRADE",IF(OR(AND(B2="SELL",E2&gt;=Parameters!$B$9),AND(B2="BUY",E2&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>NO TRADE</v>
+        <v>EXECUTED</v>
       </c>
       <c r="Q2" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="R2" s="62">
         <f t="shared" ref="R2:R21" ca="1" si="3">RAND()</f>
-        <v>0.92416331626990844</v>
+        <v>0.41563900524175212</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -2678,27 +2678,27 @@
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E21" ca="1" si="6">K2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="2">
         <f ca="1">C3-Parameters!$B$4*E3</f>
-        <v>101</v>
+        <v>100.75</v>
       </c>
       <c r="G3" s="2">
         <f ca="1">F3-Parameters!$B$3</f>
-        <v>100</v>
+        <v>99.75</v>
       </c>
       <c r="H3" s="2">
         <f ca="1">F3+Parameters!$B$3</f>
-        <v>102</v>
-      </c>
-      <c r="I3" s="2">
+        <v>101.75</v>
+      </c>
+      <c r="I3" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v/>
       </c>
       <c r="J3" s="2">
         <f t="shared" ref="J3:J21" ca="1" si="7">IF(P3&lt;&gt;"EXECUTED",J2,IF(B3="SELL",J2-I3,J2+I3))</f>
-        <v>-100</v>
+        <v>-99</v>
       </c>
       <c r="K3" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -2706,11 +2706,11 @@
       </c>
       <c r="L3" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C3-F3)))</f>
-        <v>0.5</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="N3" s="17">
         <v>0.74168005253905933</v>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="P3" s="45" t="str">
         <f ca="1">IF(R3&gt;Q3,"NO TRADE",IF(OR(AND(B3="SELL",E3&gt;=Parameters!$B$9),AND(B3="BUY",E3&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>EXECUTED</v>
+        <v>NO TRADE</v>
       </c>
       <c r="Q3" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="R3" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.24064144998442671</v>
+        <v>0.96312641995646953</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="J4" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-198.75</v>
+        <v>-197.75</v>
       </c>
       <c r="K4" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="L4" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>1.25</v>
+        <v>2.25</v>
       </c>
       <c r="M4" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C4-F4)))</f>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R4" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.56196476869988166</v>
+        <v>0.64049791962239977</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="J5" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-99.25</v>
+        <v>-98.25</v>
       </c>
       <c r="K5" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="L5" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>-0.25</v>
+        <v>0.75</v>
       </c>
       <c r="M5" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C5-F5)))</f>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="R5" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.32115760388971659</v>
+        <v>0.35521424035620608</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="J6" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-198</v>
+        <v>-197</v>
       </c>
       <c r="K6" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="L6" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C6-F6)))</f>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="R6" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.25268098784379633</v>
+        <v>4.3323104531537315E-2</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -2980,21 +2980,21 @@
         <f ca="1">F7+Parameters!$B$3</f>
         <v>99.5</v>
       </c>
-      <c r="I7" s="2" t="str">
+      <c r="I7" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>99.5</v>
       </c>
       <c r="J7" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-198</v>
+        <v>-97.5</v>
       </c>
       <c r="K7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="M7" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C7-F7)))</f>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="P7" s="45" t="str">
         <f ca="1">IF(R7&gt;Q7,"NO TRADE",IF(OR(AND(B7="SELL",E7&gt;=Parameters!$B$9),AND(B7="BUY",E7&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>NO TRADE</v>
+        <v>EXECUTED</v>
       </c>
       <c r="Q7" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="R7" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.77338633581471528</v>
+        <v>0.60957926183198718</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -3038,39 +3038,39 @@
       </c>
       <c r="E8" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="2">
         <f ca="1">C8-Parameters!$B$4*E8</f>
-        <v>99.5</v>
+        <v>99.75</v>
       </c>
       <c r="G8" s="2">
         <f ca="1">F8-Parameters!$B$3</f>
-        <v>98.5</v>
+        <v>98.75</v>
       </c>
       <c r="H8" s="2">
         <f ca="1">F8+Parameters!$B$3</f>
-        <v>100.5</v>
+        <v>100.75</v>
       </c>
       <c r="I8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>98.5</v>
+        <v>98.75</v>
       </c>
       <c r="J8" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-296.5</v>
+        <v>-196.25</v>
       </c>
       <c r="K8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>3.5</v>
+        <v>3.75</v>
       </c>
       <c r="M8" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C8-F8)))</f>
-        <v>0.6</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="N8" s="17">
         <v>0.93188989691614155</v>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="R8" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.64411270928639419</v>
+        <v>0.72903860406173593</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -3110,39 +3110,39 @@
       </c>
       <c r="E9" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" s="2">
         <f ca="1">C9-Parameters!$B$4*E9</f>
-        <v>100.25</v>
+        <v>100.5</v>
       </c>
       <c r="G9" s="2">
         <f ca="1">F9-Parameters!$B$3</f>
-        <v>99.25</v>
+        <v>99.5</v>
       </c>
       <c r="H9" s="2">
         <f ca="1">F9+Parameters!$B$3</f>
-        <v>101.25</v>
+        <v>101.5</v>
       </c>
       <c r="I9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>99.25</v>
+        <v>99.5</v>
       </c>
       <c r="J9" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-395.75</v>
+        <v>-295.75</v>
       </c>
       <c r="K9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>8.25</v>
+        <v>7.25</v>
       </c>
       <c r="M9" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C9-F9)))</f>
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="N9" s="17">
         <v>0.99516678324192342</v>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="R9" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.35267707318348274</v>
+        <v>0.36059366201691057</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -3182,39 +3182,39 @@
       </c>
       <c r="E10" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" s="2">
         <f ca="1">C10-Parameters!$B$4*E10</f>
-        <v>99</v>
+        <v>99.25</v>
       </c>
       <c r="G10" s="2">
         <f ca="1">F10-Parameters!$B$3</f>
-        <v>98</v>
+        <v>98.25</v>
       </c>
       <c r="H10" s="2">
         <f ca="1">F10+Parameters!$B$3</f>
-        <v>100</v>
+        <v>100.25</v>
       </c>
       <c r="I10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v>100.25</v>
       </c>
       <c r="J10" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-295.75</v>
+        <v>-195.5</v>
       </c>
       <c r="K10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="M10" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C10-F10)))</f>
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="N10" s="17">
         <v>0.60738987251347254</v>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="R10" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.25038237662771778</v>
+        <v>6.3292840572110376E-2</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B11" t="str">
         <f t="shared" ca="1" si="9"/>
-        <v>BUY</v>
+        <v>SELL</v>
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
@@ -3254,39 +3254,39 @@
       </c>
       <c r="E11" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" s="2">
         <f ca="1">C11-Parameters!$B$4*E11</f>
-        <v>100.25</v>
+        <v>100.5</v>
       </c>
       <c r="G11" s="2">
         <f ca="1">F11-Parameters!$B$3</f>
-        <v>99.25</v>
+        <v>99.5</v>
       </c>
       <c r="H11" s="2">
         <f ca="1">F11+Parameters!$B$3</f>
-        <v>101.25</v>
+        <v>101.5</v>
       </c>
       <c r="I11" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>101.25</v>
+        <v>99.5</v>
       </c>
       <c r="J11" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-194.5</v>
+        <v>-295</v>
       </c>
       <c r="K11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="M11" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C11-F11)))</f>
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="N11" s="17">
         <v>0.64514693645250865</v>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="R11" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>5.0335069271813637E-2</v>
+        <v>0.53047213624186573</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -3326,39 +3326,39 @@
       </c>
       <c r="E12" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="2">
         <f ca="1">C12-Parameters!$B$4*E12</f>
-        <v>101.5</v>
+        <v>101.25</v>
       </c>
       <c r="G12" s="2">
         <f ca="1">F12-Parameters!$B$3</f>
-        <v>100.5</v>
+        <v>100.25</v>
       </c>
       <c r="H12" s="2">
         <f ca="1">F12+Parameters!$B$3</f>
-        <v>102.5</v>
+        <v>102.25</v>
       </c>
       <c r="I12" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>102.5</v>
+        <v>102.25</v>
       </c>
       <c r="J12" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-92</v>
+        <v>-192.75</v>
       </c>
       <c r="K12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L12" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>11.25</v>
       </c>
       <c r="M12" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C12-F12)))</f>
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="N12" s="17">
         <v>0.30264633297266696</v>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="R12" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.72230502843196243</v>
+        <v>0.60671431295586686</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -3398,27 +3398,27 @@
       </c>
       <c r="E13" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="2">
         <f ca="1">C13-Parameters!$B$4*E13</f>
-        <v>100.75</v>
+        <v>100.5</v>
       </c>
       <c r="G13" s="2">
         <f ca="1">F13-Parameters!$B$3</f>
-        <v>99.75</v>
+        <v>99.5</v>
       </c>
       <c r="H13" s="2">
         <f ca="1">F13+Parameters!$B$3</f>
-        <v>101.75</v>
-      </c>
-      <c r="I13" s="2">
+        <v>101.5</v>
+      </c>
+      <c r="I13" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>99.75</v>
+        <v/>
       </c>
       <c r="J13" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-191.75</v>
+        <v>-192.75</v>
       </c>
       <c r="K13" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -3426,11 +3426,11 @@
       </c>
       <c r="L13" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>10.25</v>
+        <v>9.25</v>
       </c>
       <c r="M13" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C13-F13)))</f>
-        <v>0.55000000000000004</v>
+        <v>0.6</v>
       </c>
       <c r="N13" s="17">
         <v>0.78305913514582748</v>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="P13" s="45" t="str">
         <f ca="1">IF(R13&gt;Q13,"NO TRADE",IF(OR(AND(B13="SELL",E13&gt;=Parameters!$B$9),AND(B13="BUY",E13&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>EXECUTED</v>
+        <v>NO TRADE</v>
       </c>
       <c r="Q13" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="R13" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.2510777303195274</v>
+        <v>0.94512417124520121</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="J14" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-292.25</v>
+        <v>-293.25</v>
       </c>
       <c r="K14" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="L14" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>13.75</v>
+        <v>12.75</v>
       </c>
       <c r="M14" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C14-F14)))</f>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="R14" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.64348578605776752</v>
+        <v>0.41098150946321976</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
@@ -3556,21 +3556,21 @@
         <f ca="1">F15+Parameters!$B$3</f>
         <v>101.25</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>101.25</v>
+        <v/>
       </c>
       <c r="J15" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-191</v>
+        <v>-293.25</v>
       </c>
       <c r="K15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>11</v>
+        <v>9.75</v>
       </c>
       <c r="M15" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C15-F15)))</f>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="P15" s="45" t="str">
         <f ca="1">IF(R15&gt;Q15,"NO TRADE",IF(OR(AND(B15="SELL",E15&gt;=Parameters!$B$9),AND(B15="BUY",E15&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>EXECUTED</v>
+        <v>NO TRADE</v>
       </c>
       <c r="Q15" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="R15" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>6.889993461493682E-2</v>
+        <v>0.79106437065895052</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
@@ -3614,39 +3614,39 @@
       </c>
       <c r="E16" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="2">
         <f ca="1">C16-Parameters!$B$4*E16</f>
-        <v>99.5</v>
+        <v>99.25</v>
       </c>
       <c r="G16" s="2">
         <f ca="1">F16-Parameters!$B$3</f>
-        <v>98.5</v>
+        <v>98.25</v>
       </c>
       <c r="H16" s="2">
         <f ca="1">F16+Parameters!$B$3</f>
-        <v>100.5</v>
+        <v>100.25</v>
       </c>
       <c r="I16" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>98.5</v>
+        <v>98.25</v>
       </c>
       <c r="J16" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-289.5</v>
+        <v>-391.5</v>
       </c>
       <c r="K16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L16" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="M16" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C16-F16)))</f>
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="N16" s="17">
         <v>0.88926357440420511</v>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="R16" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>4.620895810152037E-2</v>
+        <v>0.21005471144722565</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
@@ -3686,39 +3686,39 @@
       </c>
       <c r="E17" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F17" s="2">
         <f ca="1">C17-Parameters!$B$4*E17</f>
-        <v>100.25</v>
+        <v>100</v>
       </c>
       <c r="G17" s="2">
         <f ca="1">F17-Parameters!$B$3</f>
-        <v>99.25</v>
+        <v>99</v>
       </c>
       <c r="H17" s="2">
         <f ca="1">F17+Parameters!$B$3</f>
-        <v>101.25</v>
+        <v>101</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>99.25</v>
+        <v>99</v>
       </c>
       <c r="J17" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-388.75</v>
+        <v>-490.5</v>
       </c>
       <c r="K17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L17" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>15.25</v>
+        <v>14.5</v>
       </c>
       <c r="M17" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C17-F17)))</f>
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="N17" s="17">
         <v>0.70612356632706164</v>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="R17" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.11333902118244221</v>
+        <v>0.71585886619021732</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
@@ -3758,31 +3758,31 @@
       </c>
       <c r="E18" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="2">
         <f ca="1">C18-Parameters!$B$4*E18</f>
-        <v>101</v>
+        <v>100.75</v>
       </c>
       <c r="G18" s="2">
         <f ca="1">F18-Parameters!$B$3</f>
-        <v>100</v>
+        <v>99.75</v>
       </c>
       <c r="H18" s="2">
         <f ca="1">F18+Parameters!$B$3</f>
-        <v>102</v>
+        <v>101.75</v>
       </c>
       <c r="I18" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>102</v>
+        <v>101.75</v>
       </c>
       <c r="J18" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-286.75</v>
+        <v>-388.75</v>
       </c>
       <c r="K18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L18" s="2">
         <f t="shared" ca="1" si="2"/>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="M18" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C18-F18)))</f>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="N18" s="17">
         <v>4.031483698143512E-2</v>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="R18" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.69103712819512142</v>
+        <v>0.39427147110892247</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
@@ -3830,39 +3830,39 @@
       </c>
       <c r="E19" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F19" s="2">
         <f ca="1">C19-Parameters!$B$4*E19</f>
-        <v>100.25</v>
+        <v>100</v>
       </c>
       <c r="G19" s="2">
         <f ca="1">F19-Parameters!$B$3</f>
-        <v>99.25</v>
+        <v>99</v>
       </c>
       <c r="H19" s="2">
         <f ca="1">F19+Parameters!$B$3</f>
-        <v>101.25</v>
+        <v>101</v>
       </c>
       <c r="I19" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>99.25</v>
+        <v>99</v>
       </c>
       <c r="J19" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-386</v>
+        <v>-487.75</v>
       </c>
       <c r="K19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>18</v>
+        <v>17.25</v>
       </c>
       <c r="M19" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C19-F19)))</f>
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="N19" s="17">
         <v>0.81169574771323405</v>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="R19" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.11015119653521888</v>
+        <v>2.9373645767939882E-2</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
@@ -3902,19 +3902,19 @@
       </c>
       <c r="E20" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F20" s="2">
         <f ca="1">C20-Parameters!$B$4*E20</f>
-        <v>99</v>
+        <v>98.75</v>
       </c>
       <c r="G20" s="2">
         <f ca="1">F20-Parameters!$B$3</f>
-        <v>98</v>
+        <v>97.75</v>
       </c>
       <c r="H20" s="2">
         <f ca="1">F20+Parameters!$B$3</f>
-        <v>100</v>
+        <v>99.75</v>
       </c>
       <c r="I20" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -3922,19 +3922,19 @@
       </c>
       <c r="J20" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-386</v>
+        <v>-487.75</v>
       </c>
       <c r="K20" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L20" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>14</v>
+        <v>12.25</v>
       </c>
       <c r="M20" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C20-F20)))</f>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="N20" s="17">
         <v>0.36539096761312051</v>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="R20" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>0.94703820705848896</v>
+        <v>0.80543592137775277</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
@@ -3974,27 +3974,27 @@
       </c>
       <c r="E21" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F21" s="2">
         <f ca="1">C21-Parameters!$B$4*E21</f>
-        <v>100</v>
+        <v>99.75</v>
       </c>
       <c r="G21" s="2">
         <f ca="1">F21-Parameters!$B$3</f>
-        <v>99</v>
+        <v>98.75</v>
       </c>
       <c r="H21" s="2">
         <f ca="1">F21+Parameters!$B$3</f>
-        <v>101</v>
-      </c>
-      <c r="I21" s="2">
+        <v>100.75</v>
+      </c>
+      <c r="I21" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v/>
       </c>
       <c r="J21" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>-485</v>
+        <v>-487.75</v>
       </c>
       <c r="K21" s="3">
         <f t="shared" ca="1" si="1"/>
@@ -4002,11 +4002,11 @@
       </c>
       <c r="L21" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>20</v>
+        <v>17.25</v>
       </c>
       <c r="M21" s="4">
         <f ca="1">MAX(0.05,MIN(0.95,0.5+Parameters!$B$7*(C21-F21)))</f>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="N21" s="17">
         <v>0.96663360539977938</v>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="P21" s="45" t="str">
         <f ca="1">IF(R21&gt;Q21,"NO TRADE",IF(OR(AND(B21="SELL",E21&gt;=Parameters!$B$9),AND(B21="BUY",E21&lt;=-Parameters!$B$9)),"REJECTED","EXECUTED"))</f>
-        <v>EXECUTED</v>
+        <v>REJECTED</v>
       </c>
       <c r="Q21" s="61">
         <f>MAX(0.05,MIN(0.95,1-Parameters!$B$10*Parameters!$B$3))</f>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="R21" s="62">
         <f t="shared" ca="1" si="3"/>
-        <v>8.9414755177511185E-2</v>
+        <v>0.17576617650190962</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
@@ -7894,7 +7894,7 @@
       <c r="C368" s="45"/>
       <c r="D368" s="49">
         <f ca="1">COUNTIF(Trades!P2:P21,"REJECTED")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E368" s="45"/>
       <c r="F368" s="45"/>

</xml_diff>